<commit_message>
Test check FA vocabulary
</commit_message>
<xml_diff>
--- a/data/raw_results/lanupro_vocabulary_fatty_acids.xlsx
+++ b/data/raw_results/lanupro_vocabulary_fatty_acids.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SH\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\my_github_projects\lanupro_vocabulary_2025\data\raw_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEA4C997-6A61-4BB5-BB82-3691C5E79B53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1414F64-FA78-44D3-9B44-C55B1F7ED516}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{06EA7712-9BA5-4E3A-B464-81F94650D082}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="596" uniqueCount="347">
   <si>
     <t>lanupro_ontology</t>
   </si>
@@ -1077,6 +1077,9 @@
   </si>
   <si>
     <t>fatty acid concentration</t>
+  </si>
+  <si>
+    <t>test</t>
   </si>
 </sst>
 </file>
@@ -2359,13 +2362,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1E034C6-174E-4BD8-87DA-20B5D61D5D37}">
-  <dimension ref="A1:BX108"/>
+  <dimension ref="A1:BY108"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="29" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:76">
+    <row r="1" spans="1:77">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2594,8 +2597,11 @@
       <c r="BX1" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="2" spans="1:76">
+      <c r="BY1" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="2" spans="1:77">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -2825,7 +2831,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="3" spans="1:76">
+    <row r="3" spans="1:77">
       <c r="A3" s="1" t="s">
         <v>111</v>
       </c>
@@ -3055,7 +3061,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="4" spans="1:76">
+    <row r="4" spans="1:77">
       <c r="A4" s="1" t="s">
         <v>266</v>
       </c>
@@ -3279,7 +3285,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="5" spans="1:76">
+    <row r="5" spans="1:77">
       <c r="A5" s="1" t="s">
         <v>112</v>
       </c>
@@ -3287,7 +3293,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="6" spans="1:76">
+    <row r="6" spans="1:77">
       <c r="A6" s="1" t="s">
         <v>113</v>
       </c>
@@ -3295,7 +3301,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="7" spans="1:76" ht="43.2">
+    <row r="7" spans="1:77" ht="43.2">
       <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
@@ -3525,7 +3531,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="8" spans="1:76">
+    <row r="8" spans="1:77">
       <c r="A8" s="1" t="s">
         <v>109</v>
       </c>
@@ -3755,42 +3761,42 @@
         <v>110</v>
       </c>
     </row>
-    <row r="9" spans="1:76">
+    <row r="9" spans="1:77">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:76">
+    <row r="10" spans="1:77">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:76">
+    <row r="11" spans="1:77">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:76">
+    <row r="12" spans="1:77">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:76">
+    <row r="13" spans="1:77">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:76">
+    <row r="14" spans="1:77">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:76">
+    <row r="15" spans="1:77">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:76">
+    <row r="16" spans="1:77">
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
Fix 2 x c18_0
</commit_message>
<xml_diff>
--- a/data/raw_results/lanupro_vocabulary_fatty_acids.xlsx
+++ b/data/raw_results/lanupro_vocabulary_fatty_acids.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\my_github_projects\lanupro_vocabulary_2025\data\raw_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1414F64-FA78-44D3-9B44-C55B1F7ED516}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CABF3E8E-DACD-4B71-A3C4-0ED5E5021B94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{06EA7712-9BA5-4E3A-B464-81F94650D082}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="596" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="345">
   <si>
     <t>lanupro_ontology</t>
   </si>
@@ -379,12 +379,6 @@
   </si>
   <si>
     <t>atol_ontology_sample_type_meat</t>
-  </si>
-  <si>
-    <t>ATOL_0000650</t>
-  </si>
-  <si>
-    <t>ATOL_0005835</t>
   </si>
   <si>
     <t>level_xx</t>
@@ -2362,231 +2356,231 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1E034C6-174E-4BD8-87DA-20B5D61D5D37}">
-  <dimension ref="A1:BY108"/>
+  <dimension ref="A1:BX108"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="29" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:77">
+    <row r="1" spans="1:76">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>2</v>
+        <v>122</v>
       </c>
       <c r="C1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D1" t="s">
         <v>124</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>125</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>126</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>127</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>128</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>129</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>130</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>131</v>
-      </c>
-      <c r="K1" t="s">
-        <v>132</v>
       </c>
       <c r="L1" t="s">
         <v>133</v>
       </c>
       <c r="M1" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="N1" t="s">
         <v>134</v>
       </c>
       <c r="O1" t="s">
+        <v>135</v>
+      </c>
+      <c r="P1" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q1" t="s">
         <v>136</v>
       </c>
-      <c r="P1" t="s">
+      <c r="R1" t="s">
         <v>137</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>140</v>
-      </c>
-      <c r="R1" t="s">
-        <v>138</v>
       </c>
       <c r="S1" t="s">
         <v>139</v>
       </c>
       <c r="T1" t="s">
+        <v>140</v>
+      </c>
+      <c r="U1" t="s">
         <v>141</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>142</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>143</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>144</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>145</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>146</v>
       </c>
       <c r="Z1" t="s">
         <v>147</v>
       </c>
       <c r="AA1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AB1" t="s">
         <v>150</v>
       </c>
       <c r="AC1" t="s">
+        <v>151</v>
+      </c>
+      <c r="AD1" t="s">
         <v>152</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AE1" t="s">
         <v>153</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AF1" t="s">
+        <v>146</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>149</v>
+      </c>
+      <c r="AH1" t="s">
         <v>154</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AI1" t="s">
         <v>155</v>
       </c>
-      <c r="AG1" t="s">
-        <v>148</v>
-      </c>
-      <c r="AH1" t="s">
-        <v>151</v>
-      </c>
-      <c r="AI1" t="s">
+      <c r="AJ1" t="s">
+        <v>2</v>
+      </c>
+      <c r="AK1" t="s">
         <v>156</v>
       </c>
-      <c r="AJ1" t="s">
+      <c r="AL1" t="s">
         <v>157</v>
       </c>
-      <c r="AK1" t="s">
-        <v>2</v>
-      </c>
-      <c r="AL1" t="s">
+      <c r="AM1" t="s">
         <v>158</v>
       </c>
-      <c r="AM1" t="s">
+      <c r="AN1" t="s">
         <v>159</v>
       </c>
-      <c r="AN1" t="s">
+      <c r="AO1" t="s">
         <v>160</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AP1" t="s">
         <v>161</v>
       </c>
-      <c r="AP1" t="s">
+      <c r="AQ1" t="s">
         <v>162</v>
       </c>
-      <c r="AQ1" t="s">
+      <c r="AR1" t="s">
         <v>163</v>
       </c>
-      <c r="AR1" t="s">
+      <c r="AS1" t="s">
         <v>164</v>
       </c>
-      <c r="AS1" t="s">
+      <c r="AT1" t="s">
         <v>165</v>
       </c>
-      <c r="AT1" t="s">
+      <c r="AU1" t="s">
         <v>166</v>
       </c>
-      <c r="AU1" t="s">
+      <c r="AV1" t="s">
         <v>167</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="AW1" t="s">
         <v>168</v>
       </c>
-      <c r="AW1" t="s">
+      <c r="AX1" t="s">
         <v>169</v>
       </c>
-      <c r="AX1" t="s">
+      <c r="AY1" t="s">
         <v>170</v>
       </c>
-      <c r="AY1" t="s">
+      <c r="AZ1" t="s">
         <v>171</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="BA1" t="s">
         <v>172</v>
       </c>
-      <c r="BA1" t="s">
+      <c r="BB1" t="s">
         <v>173</v>
-      </c>
-      <c r="BB1" t="s">
-        <v>174</v>
       </c>
       <c r="BC1" t="s">
         <v>175</v>
       </c>
       <c r="BD1" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="BE1" t="s">
         <v>176</v>
       </c>
       <c r="BF1" t="s">
+        <v>177</v>
+      </c>
+      <c r="BG1" t="s">
         <v>178</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BH1" t="s">
         <v>179</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BI1" t="s">
         <v>180</v>
       </c>
-      <c r="BI1" t="s">
+      <c r="BJ1" t="s">
         <v>181</v>
-      </c>
-      <c r="BJ1" t="s">
-        <v>182</v>
       </c>
       <c r="BK1" t="s">
         <v>183</v>
       </c>
       <c r="BL1" t="s">
+        <v>184</v>
+      </c>
+      <c r="BM1" t="s">
         <v>185</v>
       </c>
-      <c r="BM1" t="s">
+      <c r="BN1" t="s">
+        <v>182</v>
+      </c>
+      <c r="BO1" t="s">
         <v>186</v>
       </c>
-      <c r="BN1" t="s">
+      <c r="BP1" t="s">
         <v>187</v>
       </c>
-      <c r="BO1" t="s">
-        <v>184</v>
-      </c>
-      <c r="BP1" t="s">
+      <c r="BQ1" t="s">
         <v>188</v>
       </c>
-      <c r="BQ1" t="s">
+      <c r="BR1" t="s">
         <v>189</v>
       </c>
-      <c r="BR1" t="s">
+      <c r="BS1" t="s">
+        <v>337</v>
+      </c>
+      <c r="BT1" t="s">
+        <v>340</v>
+      </c>
+      <c r="BU1" t="s">
         <v>190</v>
-      </c>
-      <c r="BS1" t="s">
-        <v>191</v>
-      </c>
-      <c r="BT1" t="s">
-        <v>339</v>
-      </c>
-      <c r="BU1" t="s">
-        <v>342</v>
       </c>
       <c r="BV1" t="s">
         <v>192</v>
@@ -2595,13 +2589,10 @@
         <v>194</v>
       </c>
       <c r="BX1" t="s">
-        <v>196</v>
-      </c>
-      <c r="BY1" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="2" spans="1:77">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="2" spans="1:76">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -2827,453 +2818,447 @@
       <c r="BW2" t="s">
         <v>108</v>
       </c>
-      <c r="BX2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="3" spans="1:77">
+    </row>
+    <row r="3" spans="1:76">
       <c r="A3" s="1" t="s">
         <v>111</v>
       </c>
       <c r="B3" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="C3" t="s">
+        <v>266</v>
+      </c>
+      <c r="D3" t="s">
         <v>267</v>
-      </c>
-      <c r="D3" t="s">
-        <v>268</v>
       </c>
       <c r="E3" t="s">
         <v>269</v>
       </c>
       <c r="F3" t="s">
+        <v>270</v>
+      </c>
+      <c r="G3" t="s">
         <v>271</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>272</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
+        <v>282</v>
+      </c>
+      <c r="J3" t="s">
         <v>273</v>
       </c>
-      <c r="I3" t="s">
+      <c r="K3" t="s">
         <v>274</v>
       </c>
-      <c r="J3" t="s">
+      <c r="L3" t="s">
+        <v>283</v>
+      </c>
+      <c r="M3" t="s">
+        <v>275</v>
+      </c>
+      <c r="N3" t="s">
         <v>284</v>
       </c>
-      <c r="K3" t="s">
-        <v>275</v>
-      </c>
-      <c r="L3" t="s">
+      <c r="O3" t="s">
         <v>276</v>
       </c>
-      <c r="M3" t="s">
+      <c r="P3" t="s">
         <v>285</v>
       </c>
-      <c r="N3" t="s">
+      <c r="Q3" t="s">
+        <v>286</v>
+      </c>
+      <c r="R3" t="s">
+        <v>287</v>
+      </c>
+      <c r="S3" t="s">
         <v>277</v>
       </c>
-      <c r="O3" t="s">
-        <v>286</v>
-      </c>
-      <c r="P3" t="s">
+      <c r="T3" t="s">
+        <v>288</v>
+      </c>
+      <c r="U3" t="s">
         <v>278</v>
       </c>
-      <c r="Q3" t="s">
-        <v>287</v>
-      </c>
-      <c r="R3" t="s">
-        <v>288</v>
-      </c>
-      <c r="S3" t="s">
+      <c r="V3" t="s">
         <v>289</v>
       </c>
-      <c r="T3" t="s">
+      <c r="W3" t="s">
+        <v>290</v>
+      </c>
+      <c r="X3" t="s">
+        <v>291</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>292</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>293</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>294</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>295</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>296</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>297</v>
+      </c>
+      <c r="AE3" t="s">
         <v>279</v>
       </c>
-      <c r="U3" t="s">
-        <v>290</v>
-      </c>
-      <c r="V3" t="s">
+      <c r="AF3" t="s">
+        <v>298</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>299</v>
+      </c>
+      <c r="AH3" t="s">
+        <v>300</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>301</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>268</v>
+      </c>
+      <c r="AK3" t="s">
+        <v>302</v>
+      </c>
+      <c r="AL3" t="s">
+        <v>336</v>
+      </c>
+      <c r="AM3" t="s">
+        <v>303</v>
+      </c>
+      <c r="AN3" t="s">
+        <v>304</v>
+      </c>
+      <c r="AO3" t="s">
+        <v>305</v>
+      </c>
+      <c r="AP3" t="s">
+        <v>306</v>
+      </c>
+      <c r="AQ3" t="s">
+        <v>307</v>
+      </c>
+      <c r="AR3" t="s">
+        <v>308</v>
+      </c>
+      <c r="AS3" t="s">
+        <v>309</v>
+      </c>
+      <c r="AT3" t="s">
+        <v>310</v>
+      </c>
+      <c r="AU3" t="s">
+        <v>311</v>
+      </c>
+      <c r="AV3" t="s">
+        <v>312</v>
+      </c>
+      <c r="AW3" t="s">
+        <v>313</v>
+      </c>
+      <c r="AX3" t="s">
+        <v>314</v>
+      </c>
+      <c r="AY3" t="s">
+        <v>315</v>
+      </c>
+      <c r="AZ3" t="s">
+        <v>316</v>
+      </c>
+      <c r="BA3" t="s">
+        <v>317</v>
+      </c>
+      <c r="BB3" t="s">
+        <v>318</v>
+      </c>
+      <c r="BC3" t="s">
+        <v>319</v>
+      </c>
+      <c r="BD3" t="s">
         <v>280</v>
       </c>
-      <c r="W3" t="s">
-        <v>291</v>
-      </c>
-      <c r="X3" t="s">
-        <v>292</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>293</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>294</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>295</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>296</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>297</v>
-      </c>
-      <c r="AD3" t="s">
-        <v>298</v>
-      </c>
-      <c r="AE3" t="s">
-        <v>299</v>
-      </c>
-      <c r="AF3" t="s">
+      <c r="BE3" t="s">
+        <v>320</v>
+      </c>
+      <c r="BF3" t="s">
+        <v>321</v>
+      </c>
+      <c r="BG3" t="s">
+        <v>322</v>
+      </c>
+      <c r="BH3" t="s">
+        <v>323</v>
+      </c>
+      <c r="BI3" t="s">
+        <v>324</v>
+      </c>
+      <c r="BJ3" t="s">
+        <v>325</v>
+      </c>
+      <c r="BK3" t="s">
+        <v>326</v>
+      </c>
+      <c r="BL3" t="s">
+        <v>327</v>
+      </c>
+      <c r="BM3" t="s">
+        <v>328</v>
+      </c>
+      <c r="BN3" t="s">
         <v>281</v>
       </c>
-      <c r="AG3" t="s">
-        <v>300</v>
-      </c>
-      <c r="AH3" t="s">
-        <v>301</v>
-      </c>
-      <c r="AI3" t="s">
-        <v>302</v>
-      </c>
-      <c r="AJ3" t="s">
-        <v>303</v>
-      </c>
-      <c r="AK3" t="s">
-        <v>270</v>
-      </c>
-      <c r="AL3" t="s">
-        <v>304</v>
-      </c>
-      <c r="AM3" t="s">
+      <c r="BO3" t="s">
+        <v>329</v>
+      </c>
+      <c r="BP3" t="s">
+        <v>330</v>
+      </c>
+      <c r="BQ3" t="s">
+        <v>331</v>
+      </c>
+      <c r="BR3" t="s">
+        <v>332</v>
+      </c>
+      <c r="BS3" t="s">
         <v>338</v>
       </c>
-      <c r="AN3" t="s">
-        <v>305</v>
-      </c>
-      <c r="AO3" t="s">
-        <v>306</v>
-      </c>
-      <c r="AP3" t="s">
-        <v>307</v>
-      </c>
-      <c r="AQ3" t="s">
-        <v>308</v>
-      </c>
-      <c r="AR3" t="s">
-        <v>309</v>
-      </c>
-      <c r="AS3" t="s">
-        <v>310</v>
-      </c>
-      <c r="AT3" t="s">
-        <v>311</v>
-      </c>
-      <c r="AU3" t="s">
-        <v>312</v>
-      </c>
-      <c r="AV3" t="s">
-        <v>313</v>
-      </c>
-      <c r="AW3" t="s">
-        <v>314</v>
-      </c>
-      <c r="AX3" t="s">
-        <v>315</v>
-      </c>
-      <c r="AY3" t="s">
-        <v>316</v>
-      </c>
-      <c r="AZ3" t="s">
-        <v>317</v>
-      </c>
-      <c r="BA3" t="s">
-        <v>318</v>
-      </c>
-      <c r="BB3" t="s">
-        <v>319</v>
-      </c>
-      <c r="BC3" t="s">
-        <v>320</v>
-      </c>
-      <c r="BD3" t="s">
-        <v>321</v>
-      </c>
-      <c r="BE3" t="s">
-        <v>282</v>
-      </c>
-      <c r="BF3" t="s">
-        <v>322</v>
-      </c>
-      <c r="BG3" t="s">
-        <v>323</v>
-      </c>
-      <c r="BH3" t="s">
-        <v>324</v>
-      </c>
-      <c r="BI3" t="s">
-        <v>325</v>
-      </c>
-      <c r="BJ3" t="s">
-        <v>326</v>
-      </c>
-      <c r="BK3" t="s">
-        <v>327</v>
-      </c>
-      <c r="BL3" t="s">
-        <v>328</v>
-      </c>
-      <c r="BM3" t="s">
-        <v>329</v>
-      </c>
-      <c r="BN3" t="s">
-        <v>330</v>
-      </c>
-      <c r="BO3" t="s">
-        <v>283</v>
-      </c>
-      <c r="BP3" t="s">
-        <v>331</v>
-      </c>
-      <c r="BQ3" t="s">
-        <v>332</v>
-      </c>
-      <c r="BR3" t="s">
+      <c r="BT3" t="s">
+        <v>339</v>
+      </c>
+      <c r="BU3" t="s">
         <v>333</v>
       </c>
-      <c r="BS3" t="s">
+      <c r="BV3" t="s">
         <v>334</v>
       </c>
-      <c r="BT3" t="s">
-        <v>340</v>
-      </c>
-      <c r="BU3" t="s">
-        <v>341</v>
-      </c>
-      <c r="BV3" t="s">
+      <c r="BW3" t="s">
         <v>335</v>
       </c>
-      <c r="BW3" t="s">
-        <v>336</v>
-      </c>
-      <c r="BX3" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="4" spans="1:77">
+    </row>
+    <row r="4" spans="1:76">
       <c r="A4" s="1" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C4" t="s">
+        <v>197</v>
+      </c>
+      <c r="D4" t="s">
+        <v>198</v>
+      </c>
+      <c r="E4" t="s">
+        <v>199</v>
+      </c>
+      <c r="F4" t="s">
+        <v>200</v>
+      </c>
+      <c r="G4" t="s">
+        <v>201</v>
+      </c>
+      <c r="H4" t="s">
+        <v>202</v>
+      </c>
+      <c r="I4" t="s">
+        <v>203</v>
+      </c>
+      <c r="J4" t="s">
+        <v>204</v>
+      </c>
+      <c r="K4" t="s">
+        <v>205</v>
+      </c>
+      <c r="L4" t="s">
+        <v>206</v>
+      </c>
+      <c r="M4" t="s">
+        <v>207</v>
+      </c>
+      <c r="N4" t="s">
+        <v>208</v>
+      </c>
+      <c r="O4" t="s">
+        <v>209</v>
+      </c>
+      <c r="P4" t="s">
+        <v>210</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>211</v>
+      </c>
+      <c r="R4" t="s">
+        <v>212</v>
+      </c>
+      <c r="S4" t="s">
+        <v>213</v>
+      </c>
+      <c r="T4" t="s">
+        <v>214</v>
+      </c>
+      <c r="U4" t="s">
+        <v>215</v>
+      </c>
+      <c r="V4" t="s">
+        <v>216</v>
+      </c>
+      <c r="W4" t="s">
+        <v>217</v>
+      </c>
+      <c r="X4" t="s">
+        <v>218</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>219</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>220</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>221</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>222</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>223</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>224</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>225</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>226</v>
+      </c>
+      <c r="AG4" t="s">
+        <v>227</v>
+      </c>
+      <c r="AH4" t="s">
+        <v>228</v>
+      </c>
+      <c r="AI4" t="s">
+        <v>229</v>
+      </c>
+      <c r="AJ4" t="s">
+        <v>230</v>
+      </c>
+      <c r="AK4" t="s">
+        <v>231</v>
+      </c>
+      <c r="AL4" t="s">
         <v>232</v>
       </c>
-      <c r="C4" t="s">
-        <v>198</v>
-      </c>
-      <c r="D4" t="s">
-        <v>199</v>
-      </c>
-      <c r="E4" t="s">
-        <v>200</v>
-      </c>
-      <c r="F4" t="s">
-        <v>201</v>
-      </c>
-      <c r="G4" t="s">
-        <v>202</v>
-      </c>
-      <c r="H4" t="s">
-        <v>203</v>
-      </c>
-      <c r="I4" t="s">
-        <v>204</v>
-      </c>
-      <c r="J4" t="s">
-        <v>205</v>
-      </c>
-      <c r="K4" t="s">
-        <v>206</v>
-      </c>
-      <c r="L4" t="s">
-        <v>207</v>
-      </c>
-      <c r="M4" t="s">
-        <v>208</v>
-      </c>
-      <c r="N4" t="s">
-        <v>209</v>
-      </c>
-      <c r="O4" t="s">
-        <v>210</v>
-      </c>
-      <c r="P4" t="s">
-        <v>211</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>212</v>
-      </c>
-      <c r="R4" t="s">
-        <v>213</v>
-      </c>
-      <c r="S4" t="s">
-        <v>214</v>
-      </c>
-      <c r="T4" t="s">
-        <v>215</v>
-      </c>
-      <c r="U4" t="s">
-        <v>216</v>
-      </c>
-      <c r="V4" t="s">
-        <v>217</v>
-      </c>
-      <c r="W4" t="s">
-        <v>218</v>
-      </c>
-      <c r="X4" t="s">
-        <v>219</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>220</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>221</v>
-      </c>
-      <c r="AA4" t="s">
-        <v>222</v>
-      </c>
-      <c r="AB4" t="s">
-        <v>223</v>
-      </c>
-      <c r="AC4" t="s">
-        <v>224</v>
-      </c>
-      <c r="AD4" t="s">
-        <v>225</v>
-      </c>
-      <c r="AE4" t="s">
-        <v>226</v>
-      </c>
-      <c r="AF4" t="s">
-        <v>227</v>
-      </c>
-      <c r="AG4" t="s">
-        <v>228</v>
-      </c>
-      <c r="AH4" t="s">
-        <v>229</v>
-      </c>
-      <c r="AI4" t="s">
-        <v>230</v>
-      </c>
-      <c r="AJ4" t="s">
-        <v>231</v>
-      </c>
-      <c r="AK4" t="s">
-        <v>232</v>
-      </c>
-      <c r="AL4" t="s">
+      <c r="AM4" t="s">
         <v>233</v>
       </c>
-      <c r="AM4" t="s">
+      <c r="AN4" t="s">
         <v>234</v>
       </c>
-      <c r="AN4" t="s">
+      <c r="AO4" t="s">
         <v>235</v>
       </c>
-      <c r="AO4" t="s">
+      <c r="AP4" t="s">
         <v>236</v>
       </c>
-      <c r="AP4" t="s">
+      <c r="AQ4" t="s">
         <v>237</v>
       </c>
-      <c r="AQ4" t="s">
+      <c r="AR4" t="s">
         <v>238</v>
       </c>
-      <c r="AR4" t="s">
+      <c r="AS4" t="s">
         <v>239</v>
       </c>
-      <c r="AS4" t="s">
+      <c r="AT4" t="s">
         <v>240</v>
       </c>
-      <c r="AT4" t="s">
+      <c r="AU4" t="s">
         <v>241</v>
       </c>
-      <c r="AU4" t="s">
+      <c r="AV4" t="s">
         <v>242</v>
       </c>
-      <c r="AV4" t="s">
+      <c r="AW4" t="s">
         <v>243</v>
       </c>
-      <c r="AW4" t="s">
+      <c r="AX4" t="s">
         <v>244</v>
       </c>
-      <c r="AX4" t="s">
+      <c r="AY4" t="s">
         <v>245</v>
       </c>
-      <c r="AY4" t="s">
+      <c r="AZ4" t="s">
         <v>246</v>
       </c>
-      <c r="AZ4" t="s">
+      <c r="BA4" t="s">
+        <v>253</v>
+      </c>
+      <c r="BB4" t="s">
+        <v>254</v>
+      </c>
+      <c r="BC4" t="s">
+        <v>255</v>
+      </c>
+      <c r="BD4" t="s">
         <v>247</v>
       </c>
-      <c r="BA4" t="s">
+      <c r="BE4" t="s">
         <v>248</v>
       </c>
-      <c r="BB4" t="s">
-        <v>255</v>
-      </c>
-      <c r="BC4" t="s">
+      <c r="BF4" t="s">
+        <v>249</v>
+      </c>
+      <c r="BG4" t="s">
+        <v>250</v>
+      </c>
+      <c r="BH4" t="s">
+        <v>251</v>
+      </c>
+      <c r="BI4" t="s">
+        <v>251</v>
+      </c>
+      <c r="BJ4" t="s">
         <v>256</v>
       </c>
-      <c r="BD4" t="s">
+      <c r="BK4" t="s">
         <v>257</v>
       </c>
-      <c r="BE4" t="s">
-        <v>249</v>
-      </c>
-      <c r="BF4" t="s">
-        <v>250</v>
-      </c>
-      <c r="BG4" t="s">
-        <v>251</v>
-      </c>
-      <c r="BH4" t="s">
+      <c r="BL4" t="s">
+        <v>258</v>
+      </c>
+      <c r="BM4" t="s">
+        <v>259</v>
+      </c>
+      <c r="BN4" t="s">
         <v>252</v>
       </c>
-      <c r="BI4" t="s">
-        <v>253</v>
-      </c>
-      <c r="BJ4" t="s">
-        <v>253</v>
-      </c>
-      <c r="BK4" t="s">
-        <v>258</v>
-      </c>
-      <c r="BL4" t="s">
-        <v>259</v>
-      </c>
-      <c r="BM4" t="s">
+      <c r="BO4" t="s">
         <v>260</v>
       </c>
-      <c r="BN4" t="s">
+      <c r="BP4" t="s">
         <v>261</v>
       </c>
-      <c r="BO4" t="s">
-        <v>254</v>
-      </c>
-      <c r="BP4" t="s">
+      <c r="BQ4" t="s">
         <v>262</v>
       </c>
-      <c r="BQ4" t="s">
+      <c r="BR4" t="s">
         <v>263</v>
       </c>
-      <c r="BR4" t="s">
-        <v>264</v>
-      </c>
-      <c r="BS4" t="s">
-        <v>265</v>
+      <c r="BU4" t="s">
+        <v>191</v>
       </c>
       <c r="BV4" t="s">
         <v>193</v>
@@ -3281,257 +3266,245 @@
       <c r="BW4" t="s">
         <v>195</v>
       </c>
-      <c r="BX4" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="5" spans="1:77">
+    </row>
+    <row r="5" spans="1:76">
       <c r="A5" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B5" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="6" spans="1:77">
+    </row>
+    <row r="6" spans="1:76">
       <c r="A6" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="B6" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="7" spans="1:77" ht="43.2">
+    </row>
+    <row r="7" spans="1:76" ht="43.2">
       <c r="A7" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="P7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="Q7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="R7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="S7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="T7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="U7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="V7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="W7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="X7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="Y7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="Z7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AA7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AB7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AC7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AD7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AE7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AF7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AG7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AH7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AI7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AJ7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AK7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AL7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AM7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AN7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AO7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AP7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AQ7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AR7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AS7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AT7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AU7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AV7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AW7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AX7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AY7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="AZ7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="BA7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="BB7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="BC7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="BD7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="BE7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="BF7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="BG7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="BH7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="BI7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="BJ7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="BK7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="BL7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="BM7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="BN7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="BO7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="BP7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="BQ7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="BR7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="BS7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="BT7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="BU7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="BV7" s="3" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="BW7" s="3" t="s">
-        <v>345</v>
-      </c>
-      <c r="BX7" s="3" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="8" spans="1:77">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="8" spans="1:76">
       <c r="A8" s="1" t="s">
         <v>109</v>
       </c>
@@ -3757,46 +3730,43 @@
       <c r="BW8" t="s">
         <v>110</v>
       </c>
-      <c r="BX8" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="9" spans="1:77">
+    </row>
+    <row r="9" spans="1:76">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:77">
+    <row r="10" spans="1:76">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:77">
+    <row r="11" spans="1:76">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:77">
+    <row r="12" spans="1:76">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:77">
+    <row r="13" spans="1:76">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:77">
+    <row r="14" spans="1:76">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:77">
+    <row r="15" spans="1:76">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:77">
+    <row r="16" spans="1:76">
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
@@ -4270,7 +4240,7 @@
           <x14:formula1>
             <xm:f>description!#REF!</xm:f>
           </x14:formula1>
-          <xm:sqref>B2:BX2</xm:sqref>
+          <xm:sqref>B2:BW2</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -4323,7 +4293,7 @@
         <v>5</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -4334,7 +4304,7 @@
         <v>6</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="D3" t="s">
         <v>5</v>
@@ -4349,7 +4319,7 @@
         <v>107</v>
       </c>
       <c r="H3" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -4360,7 +4330,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="57.6">
@@ -4371,7 +4341,7 @@
         <v>5</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="57.6">
@@ -4382,7 +4352,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -4393,7 +4363,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -4404,18 +4374,18 @@
         <v>5</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B9" t="s">
         <v>5</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>